<commit_message>
Translate spread monitor workbook to English and add Macro dashboard sheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6xFB5ozPjMWRxPX9XjaG1
</commit_message>
<xml_diff>
--- a/treasury-rates-analysis-2026/ust_spread_monitor.xlsx
+++ b/treasury-rates-analysis-2026/ust_spread_monitor.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Spread Monitor" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Verdict &amp; Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chart" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Macro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Verdict &amp; Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Chart" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +68,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +88,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,11 +144,18 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -738,19 +751,19 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Treasury Spread Monitor — 2Y · 3Y · 10Y · 30Y</t>
+          <t>US Treasury Spread Monitor — 2Y / 3Y / 10Y / 30Y</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KTB 템플릿과 동일 구조 · 1Y rolling window · 작성 2026-08-29</t>
+          <t>Same layout as the KTB template · 1Y rolling window · compiled 2026-08-29</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Percentile 해석 가이드</t>
+          <t>Percentile guide</t>
         </is>
       </c>
     </row>
@@ -782,12 +795,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>(on-the-run 제네릭: GT2 Govt / GT3 Govt / GT10 Govt / GT30 Govt)</t>
+          <t>(on-the-run generics: GT2 Govt / GT3 Govt / GT10 Govt / GT30 Govt)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>0.10 = 지난 1년 중 LOWER 10% (매우 flat)</t>
+          <t>0.10 = lower 10% of past year (very flat)</t>
         </is>
       </c>
     </row>
@@ -802,7 +815,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>0.25 = LOWER 25%</t>
+          <t>0.25 = lower 25%</t>
         </is>
       </c>
     </row>
@@ -817,7 +830,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>0.50 = 중간</t>
+          <t>0.50 = middle</t>
         </is>
       </c>
     </row>
@@ -829,19 +842,19 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>FRED daily constant-maturity yields DGS2/DGS3/DGS10/DGS30 (종가, 2026-08-27까지). Bloomberg PX_LAST와 1~3bp 차이 가능. 8/28 미반영(아래 Verdict 참고).</t>
+          <t>FRED daily constant-maturity yields DGS2/DGS3/DGS10/DGS30 (closes, through 2026-08-27). May differ from Bloomberg PX_LAST by 1-3bp. Aug 28 not yet included (see Verdict sheet).</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>0.80 = HIGH 20% (already steep)</t>
+          <t>0.80 = upper 20% (already steep)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>※ 스프레드가 낮을수록(=flat) 스티프너, 높을수록(=steep) 플래트너 후보</t>
+          <t>* Low spread = flat = steepener candidate; high = steep = flattener candidate</t>
         </is>
       </c>
     </row>
@@ -878,7 +891,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>1M Δ(bp)</t>
+          <t>1M chg(bp)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -888,11 +901,11 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>해석 (1Y 기준)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>Interpretation (1Y window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>2s10s</t>
@@ -927,11 +940,11 @@
         <v/>
       </c>
       <c r="J9" s="12">
-        <f>IF(G9&lt;=0.1,"지난 1년 중 LOWER 10% (매우 flat)",IF(G9&lt;=0.25,"LOWER 25% (flat 쪽)",IF(G9&lt;0.75,"중간 범위",IF(G9&lt;0.9,"HIGH 25% (steep 쪽)","HIGH 10% (이미 매우 steep)"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
+        <f>IF(G9&lt;=0.1,"Lower 10% of past 1Y (very flat)",IF(G9&lt;=0.25,"Lower 25% (flat side)",IF(G9&lt;0.75,"Mid-range",IF(G9&lt;0.9,"Upper 25% (steep side)","Upper 10% (already very steep)"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
           <t>3s10s</t>
@@ -966,11 +979,11 @@
         <v/>
       </c>
       <c r="J10" s="12">
-        <f>IF(G10&lt;=0.1,"지난 1년 중 LOWER 10% (매우 flat)",IF(G10&lt;=0.25,"LOWER 25% (flat 쪽)",IF(G10&lt;0.75,"중간 범위",IF(G10&lt;0.9,"HIGH 25% (steep 쪽)","HIGH 10% (이미 매우 steep)"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
+        <f>IF(G10&lt;=0.1,"Lower 10% of past 1Y (very flat)",IF(G10&lt;=0.25,"Lower 25% (flat side)",IF(G10&lt;0.75,"Mid-range",IF(G10&lt;0.9,"Upper 25% (steep side)","Upper 10% (already very steep)"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>10s30s</t>
@@ -1005,11 +1018,11 @@
         <v/>
       </c>
       <c r="J11" s="12">
-        <f>IF(G11&lt;=0.1,"지난 1년 중 LOWER 10% (매우 flat)",IF(G11&lt;=0.25,"LOWER 25% (flat 쪽)",IF(G11&lt;0.75,"중간 범위",IF(G11&lt;0.9,"HIGH 25% (steep 쪽)","HIGH 10% (이미 매우 steep)"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+        <f>IF(G11&lt;=0.1,"Lower 10% of past 1Y (very flat)",IF(G11&lt;=0.25,"Lower 25% (flat side)",IF(G11&lt;0.75,"Mid-range",IF(G11&lt;0.9,"Upper 25% (steep side)","Upper 10% (already very steep)"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>2s30s</t>
@@ -1044,14 +1057,14 @@
         <v/>
       </c>
       <c r="J12" s="12">
-        <f>IF(G12&lt;=0.1,"지난 1년 중 LOWER 10% (매우 flat)",IF(G12&lt;=0.25,"LOWER 25% (flat 쪽)",IF(G12&lt;0.75,"중간 범위",IF(G12&lt;0.9,"HIGH 25% (steep 쪽)","HIGH 10% (이미 매우 steep)"))))</f>
+        <f>IF(G12&lt;=0.1,"Lower 10% of past 1Y (very flat)",IF(G12&lt;=0.25,"Lower 25% (flat side)",IF(G12&lt;0.75,"Mid-range",IF(G12&lt;0.9,"Upper 25% (steep side)","Upper 10% (already very steep)"))))</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>일별 변화 상관관계 (1Y, Δbp)</t>
+          <t>Daily-change correlation (1Y, in bp)</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1091,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>파란색 = 데이터(새 값 붙여넣기 가능) · 검정 = 수식 · 노랑 = 핵심 판정값</t>
+          <t>Blue = data (paste new values) · Black = formulas · Yellow = key outputs</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1119,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>행 추가 시 통계 범위(J24:J274 등)를 함께 조정하세요.</t>
+          <t>If you add rows, extend the stat ranges (J24:J274 etc.) accordingly.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1218,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>일별 데이터 (최신순) — 아래 표 전체가 수식 기반: 새 데이터를 위에 삽입하면 자동 재계산</t>
+          <t>Daily data (newest first) — all computed columns are formulas: insert new data on top and everything recalculates</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1235,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Δ2Y(bp)</t>
+          <t>d2Y(bp)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1232,7 +1245,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Δ3Y(bp)</t>
+          <t>d3Y(bp)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1242,7 +1255,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Δ10Y(bp)</t>
+          <t>d10Y(bp)</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -1252,7 +1265,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Δ30Y(bp)</t>
+          <t>d30Y(bp)</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -1297,22 +1310,22 @@
       </c>
       <c r="R23" s="6" t="inlineStr">
         <is>
-          <t>Δ2s10s(bp)</t>
+          <t>d2s10s(bp)</t>
         </is>
       </c>
       <c r="S23" s="6" t="inlineStr">
         <is>
-          <t>Δ3s10s(bp)</t>
+          <t>d3s10s(bp)</t>
         </is>
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>Δ10s30s(bp)</t>
+          <t>d10s30s(bp)</t>
         </is>
       </c>
       <c r="U23" s="6" t="inlineStr">
         <is>
-          <t>Δ2s30s(bp)</t>
+          <t>d2s30s(bp)</t>
         </is>
       </c>
     </row>
@@ -21626,317 +21639,874 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="95" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="95" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>스프레드 트레이드 판정 — 2026-08-27 데이터 기준 (작성 2026-08-29)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>스프레드</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Current(bp)</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Pctile</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>판정</t>
+          <t>US Macro Dashboard — Jun / Jul / Aug 2026 (by data month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Release dates in notes · compiled 2026-08-29 · sources: BLS, BEA, CNBC, Advisor Perspectives, Axios, ISM, U.Michigan, Atlanta Fed</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>3s10s</t>
-        </is>
-      </c>
-      <c r="B4" s="20">
-        <f>'Spread Monitor'!C10</f>
-        <v/>
-      </c>
-      <c r="C4" s="21">
-        <f>'Spread Monitor'!F10</f>
-        <v/>
-      </c>
-      <c r="D4" s="22">
-        <f>'Spread Monitor'!G10</f>
-        <v/>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>1Y 중 最flat (12%ile, z≈-1.3) → 통계적 스티프너 1순위. 단 3Y는 Fed 재프라이싱에 민감</t>
-        </is>
-      </c>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>INFLATION</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr"/>
+      <c r="C4" s="19" t="inlineStr"/>
+      <c r="D4" s="19" t="inlineStr"/>
+      <c r="E4" s="19" t="inlineStr"/>
+      <c r="F4" s="19" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>10s30s</t>
-        </is>
-      </c>
-      <c r="B5" s="20">
-        <f>'Spread Monitor'!C11</f>
-        <v/>
-      </c>
-      <c r="C5" s="21">
-        <f>'Spread Monitor'!F11</f>
-        <v/>
-      </c>
-      <c r="D5" s="22">
-        <f>'Spread Monitor'!G11</f>
-        <v/>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>17%ile, z≈-1.0. 재정·공급은 스팁 순풍이나 9/9~ 재무부 장기물 바이백이 30Y 지지 → 역풍 공존</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>2s30s</t>
-        </is>
-      </c>
-      <c r="B6" s="20">
-        <f>'Spread Monitor'!C12</f>
-        <v/>
-      </c>
-      <c r="C6" s="21">
-        <f>'Spread Monitor'!F12</f>
-        <v/>
-      </c>
-      <c r="D6" s="22">
-        <f>'Spread Monitor'!G12</f>
-        <v/>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>20%ile, z≈-0.8. 방향은 같으나 vol(3.6bp/d) 최대 → 사이즈 유의</t>
+          <t>CPI headline</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>-0.4%</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>+0.1%</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>due ~Sep 10</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Jun: largest monthly drop since Apr 2020; beat 3.8% y/y consensus. Released Jul 14 / Aug 12.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>2s10s</t>
-        </is>
-      </c>
-      <c r="B7" s="20">
-        <f>'Spread Monitor'!C9</f>
-        <v/>
-      </c>
-      <c r="C7" s="21">
-        <f>'Spread Monitor'!F9</f>
-        <v/>
-      </c>
-      <c r="D7" s="22">
-        <f>'Spread Monitor'!G9</f>
-        <v/>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>22%ile, z≈-0.6 → 중립~약한 스티프너. 신호 강도 부족</t>
+      <c r="A7" s="12" t="inlineStr"/>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>3.5%</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>3.4%</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Peaked at 4.2% in May (Iran war / oil shock); easing but stuck in the 3s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Core CPI</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>due ~Sep 10</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Core is well-behaved — the problem is energy.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>종합 판정</t>
-        </is>
-      </c>
+      <c r="A9" s="12" t="inlineStr"/>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>2.6%</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>· 4개 스프레드 모두 1Y 하위 25% (flat 쪽) — 평균회귀 관점의 방향은 "스티프너"이나, |z|&lt;1.5로 극단 아님 → "괜찮지만 아직 싸지 않다".</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>PCE headline</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>-0.1%</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>due late Sep</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Jul beat +0.1% consensus. Released Jul 31 / Aug 26.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>· 이번 여름 flat화의 원인이 명확: 8/28 Warsh 잭슨홀 매파 발언으로 2Y +6bp(4.34%), 9월 인상확률 35%→58% (CME). 인상 현실화 시 bear-flattening 추가 진행 위험.</t>
+      <c r="A11" s="12" t="inlineStr"/>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>3.7%</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>3.7%</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>Eased from 4.1% in May, then stalled — disinflation paused.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>· 참고: 8/28 종가(FRED 미반영)는 2Y 4.34 / 10Y 4.73 / 30Y 5.17 → 2s10s ≈39bp (z≈-1.4), 10s30s ≈44bp (z≈-2.3, 1Y 최저) — 진입 레벨은 더 매력적, 촉매 리스크는 더 커짐.</t>
-        </is>
-      </c>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Core PCE</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>+0.1%</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>due late Sep</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>· 실행안: (1) 9/16 FOMC 전 절반, 이후 절반 분할 진입  (2) 10s30s 스티프너는 바이백(9/9~11/4, 회당 ≥$40억) 종료 전까지 보수적으로  (3) 손절 기준: z가 -2.5 이탈 또는 인상 사이클 본격화.</t>
+      <c r="A13" s="12" t="inlineStr"/>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>3.3%</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>3.3%</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>Above 3.2% consensus; 1.3pp over the 2% target and going sideways — the hawks' key exhibit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>PPI headline</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>due ~Sep 10</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>Jul flat vs +0.2% expected. Released Jul 15 / Aug 13.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>촉매 캘린더</t>
+      <c r="A15" s="12" t="inlineStr"/>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>5.5%</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>4.7%</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>Down from 6.0% in May — pipeline pressure cooling fast.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>9/2~4 고용지표 · 9/9 바이백 개시 · 9/10경 CPI · 9/16 FOMC(인상확률 ~58%) · 10월 refunding · 이란/유가, 재정적자(7월 $432B), 국채발행 $739B(Q3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>DV01 중립 헤지비율 (근사 — 실제는 단말 DV01 사용)</t>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Core PPI</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>+0.4%</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>+0.2%</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>due ~Sep 10</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Jul below 0.3% consensus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr"/>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>n/a*</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>*Jul y/y conflicting across sources (a reported 4.2% looks like the ex-food/energy/trade series) — verify on terminal.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>만기</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>근사 듀레이션</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>DV01/100mm</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>스티프너 예: 10Y 100mm 매도 대비 매수 notional</t>
-        </is>
-      </c>
+          <t>LABOR</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr"/>
+      <c r="C19" s="19" t="inlineStr"/>
+      <c r="D19" s="19" t="inlineStr"/>
+      <c r="E19" s="19" t="inlineStr"/>
+      <c r="F19" s="19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="C20" s="25">
-        <f>B20/100*10000</f>
-        <v/>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>2s10s: 2Y ≈ 100mm × C22/C20 ≈ 416mm 매수</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="C21" s="25">
-        <f>B21/100*10000</f>
-        <v/>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>3s10s: 3Y ≈ 100mm × C22/C21 ≈ 282mm 매수</t>
+          <t>Nonfarm payrolls</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>k, m/m</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>+57k -&gt; revised +20k</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>-23k (exp +80k)</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 4</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>Jul: first negative print; two-month revisions -103k. Released Jul 2 / Aug 7.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B22" s="24" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="C22" s="25">
-        <f>B22/100*10000</f>
-        <v/>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>10s30s: 30Y 매도 시 10Y ≈ 30Y notional × C23/C22 ≈ 2.03배 매수</t>
+          <t>Unemployment rate</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>4.2%</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>4.1%</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 4</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Fell for the wrong reason: participation 61.4%, a 5-year low (labor supply shrinking).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>30Y</t>
-        </is>
-      </c>
-      <c r="B23" s="24" t="n">
-        <v>16</v>
-      </c>
-      <c r="C23" s="25">
-        <f>B23/100*10000</f>
-        <v/>
-      </c>
-      <c r="D23" s="26" t="inlineStr">
-        <is>
-          <t>(가격·수익률 수준 따라 변동 — 근사치)</t>
+          <t>Avg hourly earnings</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>y/y</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>+3.2%</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 4</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>Slowest since May 2021 — wage-push pressure fading.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23">
-        <f>BDH("USGG2YR Index","PX_LAST","8/27/2025","","Dir=V","Dts=S","Sort=D")  ← Date+PX_LAST 세로 출력, 최신순</f>
-        <v/>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>ADP private payrolls</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>k, m/m</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>+95k (rev.)</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>+44k (exp +70k)</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 2</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Hiring slowdown confirmed.</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>티커: USGG2YR/USGG3YR/USGG10YR/USGG30YR Index (제네릭 수익률) 또는 GT2/GT3/GT10/GT30 Govt. KTB의 GTKRW#YR Corp와 동일 계열은 GT# Govt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>붙여넣기: Spread Monitor 시트 B/D/F/H열(파란색)에 값만 교체 — 스프레드·Z·백분위 전부 자동 재계산.</t>
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Initial jobless claims</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>~190k</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>low-200k</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>203k (wk Aug 22)</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>Near 60-year lows — no layoffs; a hiring freeze, not a firing cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>ACTIVITY &amp; EXPECTATIONS</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr"/>
+      <c r="C27" s="19" t="inlineStr"/>
+      <c r="D27" s="19" t="inlineStr"/>
+      <c r="E27" s="19" t="inlineStr"/>
+      <c r="F27" s="19" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Retail sales</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>m/m</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>+0.2% (+6.7% y/y)</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>-0.6% (+5.0% y/y)</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>due mid-Sep</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <t>Jul: biggest drop in over a year — consumer breather.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>ISM Manufacturing</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>53.3</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>55.6</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 1</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>Jul highest since May 2022; Aug S&amp;P flash mfg 53.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>ISM Services</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>54.1</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>due Sep 3</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <t>Aug S&amp;P flash services 56.8, composite 56.0 (best since Apr 2022).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Real GDP</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>saar</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Q2 +1.5%</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>GDPNow Q3: 4.6%</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>Q2 second estimate unchanged; consumption revised up to +3.4%. GDPNow as of Aug 26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>U.Mich inflation exp.</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>1y / 5-10y</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>4.6% / 3.3%</t>
+        </is>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>4.2% / 3.3%</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="inlineStr">
+        <is>
+          <t>4.3% / 3.3% (prelim)</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <t>Long-run expectations anchored at 3.3%; Aug sentiment 51.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>TAKEAWAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>Inflation: headline stuck in the 3s, core PCE flat at 3.3% — no progress toward 2% since June.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>Labor: cooling sharply, but via shrinking supply (participation), not layoffs — claims near 60-yr lows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>Activity: re-accelerating (GDPNow 4.6%, flash PMI 56.0, record-adjacent equities).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>Net: the Fed cannot cut (Sep 16 hike odds ~58% post-Jackson Hole); growth supports real yields; inflation uncertainty feeds the term premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>Event calendar: Sep 2 ADP · Sep 4 NFP · Sep 9 Treasury buybacks start · ~Sep 10 CPI/PPI · Sep 16 FOMC.</t>
         </is>
       </c>
     </row>
@@ -21951,13 +22521,338 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Spread Trade Verdict — data through 2026-08-27 (compiled 2026-08-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Current(bp)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Pctile</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>3s10s</t>
+        </is>
+      </c>
+      <c r="B4" s="24">
+        <f>'Spread Monitor'!C10</f>
+        <v/>
+      </c>
+      <c r="C4" s="25">
+        <f>'Spread Monitor'!F10</f>
+        <v/>
+      </c>
+      <c r="D4" s="26">
+        <f>'Spread Monitor'!G10</f>
+        <v/>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Flattest of the past 1Y (12th pctile, z ~ -1.3) -&gt; strongest statistical steepener candidate. Note the 3Y is the most sensitive point to Fed repricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>10s30s</t>
+        </is>
+      </c>
+      <c r="B5" s="24">
+        <f>'Spread Monitor'!C11</f>
+        <v/>
+      </c>
+      <c r="C5" s="25">
+        <f>'Spread Monitor'!F11</f>
+        <v/>
+      </c>
+      <c r="D5" s="26">
+        <f>'Spread Monitor'!G11</f>
+        <v/>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>17th pctile, z ~ -1.0. Fiscal/supply argues steeper, but Treasury long-end buybacks from Sep 9 support the 30Y -&gt; crosswinds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>2s30s</t>
+        </is>
+      </c>
+      <c r="B6" s="24">
+        <f>'Spread Monitor'!C12</f>
+        <v/>
+      </c>
+      <c r="C6" s="25">
+        <f>'Spread Monitor'!F12</f>
+        <v/>
+      </c>
+      <c r="D6" s="26">
+        <f>'Spread Monitor'!G12</f>
+        <v/>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>20th pctile, z ~ -0.8. Same direction, but highest vol (3.6bp/d) -&gt; size accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2s10s</t>
+        </is>
+      </c>
+      <c r="B7" s="24">
+        <f>'Spread Monitor'!C9</f>
+        <v/>
+      </c>
+      <c r="C7" s="25">
+        <f>'Spread Monitor'!F9</f>
+        <v/>
+      </c>
+      <c r="D7" s="26">
+        <f>'Spread Monitor'!G9</f>
+        <v/>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>22nd pctile, z ~ -0.6 -&gt; neutral-to-mild steepener. Signal not strong enough on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Overall verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>- All four spreads sit in the lower 12-22% of their 1Y range (flat side) — mean-reversion favors STEEPENERS, but |z| &lt; 1.5, so "decent, not yet cheap".</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>- The flattening has a clear cause: Warsh's hawkish Jackson Hole speech (Aug 28) pushed the 2Y to 4.34% and Sept hike odds from 35% to ~58% (CME). If a hike lands, bear-flattening can extend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>- Note: Aug 28 closes (not yet in FRED data): 2Y 4.34 / 10Y 4.73 / 30Y 5.17 -&gt; 2s10s ~39bp (z ~ -1.4), 10s30s ~44bp (z ~ -2.3, 1Y low) — better entry levels, bigger catalyst risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>- Execution: (1) scale in half before / half after the Sep 16 FOMC  (2) be conservative on 10s30s steepeners until buybacks end (Sep 9 - Nov 4, &gt;= $4bn per op)  (3) stop-loss: z breaks below -2.5 or a genuine hiking cycle starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Catalyst calendar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Sep 2-4 labor data · Sep 9 buybacks start · ~Sep 10 CPI · Sep 16 FOMC (hike odds ~58%) · October refunding · Iran/oil, fiscal deficit (Jul $432bn), $739bn Q3 borrowing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>DV01-neutral hedge ratios (approximate — use terminal DV01 for execution)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Approx duration</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>DV01 / 100mm</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Steepener example vs 100mm 10Y short</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C20" s="28">
+        <f>B20/100*10000</f>
+        <v/>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>2s10s: buy ~ 100mm x C22/C20 ~ 416mm of 2Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C21" s="28">
+        <f>B21/100*10000</f>
+        <v/>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>3s10s: buy ~ 100mm x C22/C21 ~ 282mm of 3Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C22" s="28">
+        <f>B22/100*10000</f>
+        <v/>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>10s30s: per 100mm 30Y short, buy ~ C23/C22 ~ 2.0x notional of 10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>30Y</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="C23" s="28">
+        <f>B23/100*10000</f>
+        <v/>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>(Approximations — vary with price/yield level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22">
+        <f>BDH("USGG2YR Index","PX_LAST","8/27/2025","","Dir=V","Dts=S","Sort=D")   &lt;- Date + PX_LAST, vertical, newest first</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>Tickers: USGG2YR / USGG3YR / USGG10YR / USGG30YR Index (generic yields) or GT2 / GT3 / GT10 / GT30 Govt. The US equivalent of KTB's GTKRW#YR Corp series is GT# Govt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Paste values into the blue columns (B/D/F/H) of the Spread Monitor sheet — spreads, Z-scores and percentiles all recalculate automatically.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>스프레드 추이 (bp, 1Y)</t>
+          <t>Spread history (bp, 1Y)</t>
         </is>
       </c>
     </row>

</xml_diff>